<commit_message>
push2desktop update attach_sensors function
</commit_message>
<xml_diff>
--- a/shipClassTests/testResults/system_example.xlsx
+++ b/shipClassTests/testResults/system_example.xlsx
@@ -479,7 +479,7 @@
         <v>2</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -496,16 +496,16 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4">
         <v>2</v>
@@ -519,16 +519,16 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5">
         <v>2</v>
@@ -542,16 +542,16 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6">
         <v>2</v>
@@ -565,16 +565,16 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7">
         <v>2</v>
@@ -588,10 +588,10 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -611,10 +611,10 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -634,10 +634,10 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C10">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -657,16 +657,16 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C11">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F11">
         <v>2</v>
@@ -680,10 +680,10 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C12">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -703,10 +703,10 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -729,13 +729,13 @@
         <v>0</v>
       </c>
       <c r="C14">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D14">
         <v>0</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F14">
         <v>2</v>
@@ -752,16 +752,16 @@
         <v>0</v>
       </c>
       <c r="C15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D15">
         <v>0</v>
       </c>
       <c r="E15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G15" s="4">
         <v>2</v>
@@ -775,16 +775,16 @@
         <v>0</v>
       </c>
       <c r="C16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D16">
         <v>0</v>
       </c>
       <c r="E16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G16" s="4">
         <v>2</v>
@@ -798,16 +798,16 @@
         <v>0</v>
       </c>
       <c r="C17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D17">
         <v>0</v>
       </c>
       <c r="E17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G17" s="4">
         <v>2</v>
@@ -821,16 +821,16 @@
         <v>0</v>
       </c>
       <c r="C18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D18">
         <v>0</v>
       </c>
       <c r="E18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G18" s="4">
         <v>2</v>
@@ -844,16 +844,16 @@
         <v>0</v>
       </c>
       <c r="C19">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D19">
         <v>0</v>
       </c>
       <c r="E19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G19" s="4">
         <v>2</v>
@@ -867,16 +867,16 @@
         <v>0</v>
       </c>
       <c r="C20">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D20">
         <v>0</v>
       </c>
       <c r="E20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G20" s="4">
         <v>2</v>
@@ -890,16 +890,16 @@
         <v>0</v>
       </c>
       <c r="C21">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D21">
         <v>0</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21" s="4">
         <v>2</v>
@@ -913,16 +913,16 @@
         <v>0</v>
       </c>
       <c r="C22">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D22">
         <v>0</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22" s="4">
         <v>2</v>
@@ -936,16 +936,16 @@
         <v>0</v>
       </c>
       <c r="C23">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D23">
         <v>0</v>
       </c>
       <c r="E23">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F23">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G23" s="4">
         <v>2</v>
@@ -959,16 +959,16 @@
         <v>0</v>
       </c>
       <c r="C24">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D24">
         <v>0</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F24">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G24" s="4">
         <v>2</v>
@@ -982,16 +982,16 @@
         <v>0</v>
       </c>
       <c r="C25">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D25">
         <v>0</v>
       </c>
       <c r="E25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G25" s="4">
         <v>2</v>
@@ -1005,16 +1005,16 @@
         <v>0</v>
       </c>
       <c r="C26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D26">
         <v>0</v>
       </c>
       <c r="E26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F26">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G26" s="4">
         <v>2</v>
@@ -1028,13 +1028,13 @@
         <v>0</v>
       </c>
       <c r="C27">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D27">
         <v>0</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F27">
         <v>0</v>
@@ -1125,7 +1125,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1133,7 +1133,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1141,7 +1141,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1149,7 +1149,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1157,7 +1157,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -1165,7 +1165,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -1173,7 +1173,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -1181,7 +1181,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -1189,7 +1189,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -1197,7 +1197,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -1205,7 +1205,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -1213,7 +1213,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -1221,7 +1221,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -1229,7 +1229,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -1237,7 +1237,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -1245,7 +1245,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -1253,7 +1253,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -1261,7 +1261,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -1269,7 +1269,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -1277,7 +1277,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -1285,7 +1285,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -1293,7 +1293,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -1301,7 +1301,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -1309,7 +1309,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1346,7 +1346,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1354,7 +1354,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1362,7 +1362,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1370,7 +1370,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1378,7 +1378,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1583,7 +1583,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1591,7 +1591,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1599,7 +1599,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1607,7 +1607,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1639,7 +1639,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -1663,7 +1663,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -1671,7 +1671,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -1679,7 +1679,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -1687,7 +1687,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -1695,7 +1695,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -1703,7 +1703,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -1711,7 +1711,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -1719,7 +1719,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -1727,7 +1727,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -1735,7 +1735,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -1743,7 +1743,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -1751,7 +1751,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -1759,7 +1759,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -1767,7 +1767,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1900,7 +1900,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -1908,7 +1908,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -1916,7 +1916,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -1924,7 +1924,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -1932,7 +1932,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -1940,7 +1940,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -1948,7 +1948,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -1956,7 +1956,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -1964,7 +1964,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -1972,7 +1972,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -1980,7 +1980,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -1988,7 +1988,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:2">

</xml_diff>